<commit_message>
Rebuild site from updated 叫序表 source data
Picks up content edits in the five bidding-table workbooks, including
第十一章 revision content: 一方塊開叫.xlsx gains a "13.第十一章修訂"
sheet (with a deprecated "F舊" branch kept for reference in the F-J
merged sheet) and 一梅花開叫.xlsx gains "14.第十一章改動1". Renumbered
一梅花被插叫.xlsx's merged sheets from 14-17 to 15-18 since the new
sheet 14 in 一梅花開叫.xlsx would otherwise collide with it and break
the "見表14" cross-reference in 12.(原)1♣–2♠系統. Updated the stale
homepage worksheet counts (一方塊開叫 12→13, 一梅花開叫 18→19).
Verified zero broken links/anchors across the rebuilt site.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S7A2DTuvm4TLYq1CrLS1wj
</commit_message>
<xml_diff>
--- a/原始資料/一方塊開叫.xlsx
+++ b/原始資料/一方塊開叫.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10.非接力叫牌" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11.示例牌張" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12.示例叫序" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13.第十一章修訂" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +75,12 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -103,7 +110,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -125,11 +132,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -207,6 +258,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -572,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -608,348 +664,415 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>開叫定義</t>
+          <t>★ 家規點力</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>1♦ = 至少一張♦ + 11-15大牌點。含義甚廣的多功能開叫，三種典型牌型：①至少5張♦的非均型牌　②均型牌但點力不在1NT範圍　③雙低花套（6♣+5♦ 總是開1♦，有時6♣+4♦ 也開1♦）。</t>
+          <t>本檔採用家規點力：**所有開叫點力下修 1 點、所有答叫點力上修 1 點**（聯手總點力因此維持不變）。括號內或註明「原書」者為原書印行的數值。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>接力扳機</t>
+          <t>開叫定義</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>1♥。這一叫品是雙重含義：接力序列（逼叫進局）的開始，或至少4張♥+6點以上的自然叫。</t>
+          <t>1♦ = 至少一張♦ + 10-14大牌點（家規下修 1 點；原書 11-15）。**低限 = 10-12 點，高限 = 13-14 點。**含義甚廣的多功能開叫，三種典型牌型：①至少5張♦的非均型牌　②均型牌但點力不在1NT範圍　③雙低花套（6♣+5♦ 總是開1♦，有時6♣+4♦ 也開1♦）。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>核心設計</t>
+          <t>接力扳機</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>開叫者的第一次再叫「總是先假定 1♥ 是自然叫」，在這個假定上描述牌型。因此僅有三張♥支持時不能直接加叫。</t>
+          <t>1♥。這一叫品是雙重含義：接力序列（逼叫進局）的開始，或至少4張♥+7點以上的自然叫。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>核心設計</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>開叫者的第一次再叫「總是先假定 1♥ 是自然叫」，在這個假定上描述牌型。因此僅有三張♥支持時不能直接加叫。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>牌型寫法</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>四位數字一律按 ♠-♥-♦-♣ 順序。例：3-3-7-0 是 7張♦、♣缺門。</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>接力術語</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>說明</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>接力（Relay）</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>最便宜的叫品，要求同伴繼續描述牌型。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Sidestep</t>
+          <t>接力（Relay）</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>問「剩下兩門怎麼分」。由平均排到極端，同程度時級別較高的那門較短排前面。</t>
+          <t>最便宜的叫品，要求同伴繼續描述牌型。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Splinter-relay</t>
+          <t>Sidestep</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>問「短套在哪門」。三級，由最低級花色排到最高級。</t>
+          <t>問「剩下兩門怎麼分」。由平均排到極端，同程度時級別較高的那門較短排前面。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>54Pick-up</t>
+          <t>Splinter-relay</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>問 5-4 牌型中那個 4 張套在哪一門、幾張。</t>
+          <t>問「短套在哪門」。三級，由最低級花色排到最高級。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Six-shooter</t>
+          <t>54Pick-up</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>問 6 張以上單套牌的完整分佈，七級一次講完。</t>
+          <t>問 5-4 牌型中那個 4 張套在哪一門、幾張。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>Six-shooter</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>問 6 張以上單套牌的完整分佈，七級一次講完。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>CRASH</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>牌型問完後問 A、K、Q 的確切位置（Colour-Rank-And-SHape）。</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
-      <c r="B17" s="5" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>本章特有規則</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>說明</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>4♠ 上限</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>4♠ 是詢問牌型的接力中最高階次的叫品。H分支 4♠ 之後的 4NT 是黑木，不是接力。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>成局線上的止叫</t>
+          <t>4♠ 上限</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>任何在成局線上、且同伴至少保證四張的叫品都是止叫。J分支 4♥ 之後只能用 4NT 做 CRASH。</t>
+          <t>4♠ 是詢問牌型的接力中最高階次的叫品。H分支 4♠ 之後的 4NT 是黑木，不是接力。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>C分支的加一級</t>
+          <t>成局線上的止叫</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>C分支前五個答叫多插一級：第一級答叫表示低限，下一次接力才是普通的 Sidestep。</t>
+          <t>任何在成局線上、且同伴至少保證四張的叫品都是止叫。J分支 4♥ 之後只能用 4NT 做 CRASH。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
+          <t>C分支的加一級</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>C分支前五個答叫多插一級：第一級答叫表示低限，下一次接力才是普通的 Sidestep。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>巢狀子接力</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>A分支的 2♦ 和 E分支的 3♣／3♦ 底下各自還有一層獨立接力，本檔用縮排與底色區分。</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
-      <c r="B23" s="5" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>工作表</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>內容</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>2. 第一應叫</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>開叫 1♦ 後應叫者的全部應叫及含義。</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>3. 接力主幹</t>
+          <t>2. 第一應叫</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>1♦ – 1♥ 後，開叫者的 14 種再叫與對應接力叫品。</t>
+          <t>開叫 1♦ 後應叫者的全部應叫及含義。</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>4. A分支（1♠）</t>
+          <t>3. 接力主幹</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>1♠ = 4張♠否認4張♥。5種再叫，含 2♦ 的巢狀子接力。</t>
+          <t>1♦ – 1♥ 後，開叫者的 14 種再叫與對應接力叫品。</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>5. B分支（1NT）</t>
+          <t>4. A分支（1♠）</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>1NT = 均型牌無四張高花。6種再叫。</t>
+          <t>1♠ = 4張♠否認4張♥。5種再叫，含 2♦ 的巢狀子接力。</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>6. C分支（2♣）</t>
+          <t>5. B分支（1NT）</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2♣ = 低花上至少9張牌。8種再叫。</t>
+          <t>1NT = 均型牌無四張高花。6種再叫。</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>7. D分支（2♦）</t>
+          <t>6. C分支（2♣）</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>2♦ = 6張以上♦無邊花套。7種再叫（Six-shooter）。</t>
+          <t>2♣ = 低花上至少9張牌。8種再叫。</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>8. E分支（2♥）</t>
+          <t>7. D分支（2♦）</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2♥ = 4張♥。6種再叫，含兩組巢狀子接力。</t>
+          <t>2♦ = 6張以上♦無邊花套。7種再叫（Six-shooter）。</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>9. F-J分支</t>
+          <t>8. E分支（2♥）</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>F～J 五個高限與爆裂叫分支合併於一表。</t>
+          <t>2♥ = 4張♥。6種再叫，含兩組巢狀子接力。</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>10. 非接力叫牌</t>
+          <t>9. F-J分支</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>應叫者實力不夠逼叫到局時的自然叫進程。</t>
+          <t>F～J 五個高限與爆裂叫分支合併於一表。</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>11. 示例牌張</t>
+          <t>10. 非接力叫牌</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>例1–例6 的持牌、局況與結果評論。</t>
+          <t>應叫者實力不夠逼叫到局時的自然叫進程。</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
+          <t>11. 示例牌張</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>例1–例6 的持牌、局況與結果評論。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
           <t>12. 示例叫序</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>例1–例6 的完整叫序，逐叫列出。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>13. 第十一章修訂</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>★ 第十一章對本章的四處改寫（修訂A–D）新舊對照。表3、4、8、9 均已就地更新。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr"/>
+      <c r="B38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>★ 第十一章的影響</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>說明</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>為什麼要改</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>第十一章新增了「2♦ ＝ 4-8點、5張高花+4張低花」的選擇性開叫。這使得 4-4-4-1 牌型不得不全部歸給 1♦ 開叫，原有的接力設計容納不下，因此有了修訂 A～D 四處改寫。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>改了哪四處</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>A：表3／表9 的 F分支 2♠ 改為「4441、有4張♥、高限」。
+B：表4 A分支的 2♠ 改為「4張♠+1或2張♥」，收 4-1-4-4。
+C：表8 E分支的 2NT 改為「4張♥+4張♠」，收 4-4-1-4／4-4-4-1（低限）。
+D：表8 E分支 3♣ 的階梯改寫，插入 1-4-4-4（低限）。</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1202,7 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>簡單加叫，8-11大牌點，通常4張♠支持和至少4張♥</t>
+          <t>簡單加叫，9-12大牌點，通常4張♠支持和至少4張♥</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1941,7 +2064,7 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>均型牌，無四張高花，13-15大牌點（B分支）</t>
+          <t>均型牌，無四張高花，13-14大牌點（B分支）</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3280,7 @@
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>均型牌，無4張高花，11-13點（B分支）</t>
+          <t>均型牌，無4張高花，10-12點（B分支）</t>
         </is>
       </c>
     </row>
@@ -3594,6 +3717,561 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A64:F64"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>第十一章對第四章的四處修訂</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>起因：第十一章新增「2♦ ＝ 4-8點、5張高花+4張低花」的選擇性開叫，4-4-4-1 牌型因而全部歸於 1♦ 開叫</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>修訂</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>序列</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>叫品</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>原含義（已作廢）</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>新含義</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>1♦–1♥；2♠–2NT；？　（表3 F分支／表9）</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>2♠</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>4張以上♠ + 5張以上♦，高限</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>4-4-4-1牌型，有4張♥，高限</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>1♦–1♥；1♠–2♣；2♠–2NT；？　（表4 A分支）</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>2♠</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>2張♥，低花 3-4 或 4-3</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>4張♠ + 1或2張♥</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>1♦–1♥；2♥–2♠；2NT–3♣；？　（表8 E分支）</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>2NT</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>4張♠</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>4張♥ + 4張♠</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>1♦–1♥；2♥–2♠；3♣–3♦；？　（表8 E分支）</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>3♣</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>4張♥ + 4張以上♣（叫品含義不變，改的是答叫階梯）</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>4張♥ + 4張以上♣（階梯改寫，見下）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>修訂 A　1♦ – 1♥；2♠ – 2NT；？　（2♠ ＝ 4-4-4-1，有4張♥，高限）</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="n"/>
+      <c r="C10" s="30" t="n"/>
+      <c r="D10" s="30" t="n"/>
+      <c r="E10" s="31" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr"/>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>3♣</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>4-4-4-1，高限（♣單張）</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>3♦ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr"/>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>3♦</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr"/>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>4-4-1-4，高限（♦單張）</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>3♥ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr"/>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>3♥</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>1-4-4-4，高限（♠單張）</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>3♠ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>註：三個答叫都含4張♥，所以 4-1-4-4（♥單張）不在此列——那一型改由修訂 B 處理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>修訂 B　1♦ – 1♥；1♠ – 2♣；2♠ – 2NT；？　（2♠ ＝ 4張♠ + 1或2張♥）</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="n"/>
+      <c r="C16" s="30" t="n"/>
+      <c r="D16" s="30" t="n"/>
+      <c r="E16" s="31" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr"/>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>3♣</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr"/>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>4-2-3-4</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>3♦ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr"/>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>3♦</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr"/>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>4-2-4-3</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>3♥ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr"/>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>3♥</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr"/>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>4-1-4-4，低限</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>3♠ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr"/>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>3♠</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr"/>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>4-1-4-4，高限</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>4♣ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>註：前兩級是原本就有的 4-2-x-x，後兩級是新收進來的 4441（♥單張），用低限／高限分兩級。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>修訂 C　1♦ – 1♥；2♥ – 2♠；2NT – 3♣；？　（2NT ＝ 4張♥ + 4張♠）</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="n"/>
+      <c r="C23" s="30" t="n"/>
+      <c r="D23" s="30" t="n"/>
+      <c r="E23" s="31" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr"/>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>3♦</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr"/>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>4-4-2-3</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>3♥ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr"/>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>3♥</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr"/>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>4-4-3-2</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>3♠ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr"/>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>3♠</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr"/>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>4-4-1-4，低限</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>4♣ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr"/>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>3NT</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr"/>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>4-4-4-1，低限</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>4♣ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="28" t="inlineStr">
+        <is>
+          <t>註：階梯符合通則：先問「剩兩門怎麼分」由平均到極端（2-3 → 3-2 → 1-4 → 4-1）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>修訂 D　1♦ – 1♥；2♥ – 2♠；3♣ – 3♦；？　（3♣ ＝ 4張♥ + 4張以上♣）</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="n"/>
+      <c r="C30" s="30" t="n"/>
+      <c r="D30" s="30" t="n"/>
+      <c r="E30" s="31" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr"/>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>3♥</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr"/>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>2-4-3-4</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>3♠ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr"/>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>3♠</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr"/>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>3-4-2-4</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>4♣ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr"/>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>3NT</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr"/>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>1-4-4-4，低限　← 新插入</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>4♣ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr"/>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>4♣</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr"/>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>2-4-2-5　← 原為第3級，順延一級</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>4♦ = CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="28" t="inlineStr">
+        <is>
+          <t>註：原設計為：3♥=2-4-3-4、3♠=3-4-2-4、3NT=2-4-2-5、4♣=1-4-3-5、4♦=3-4-1-5。新版取消 1-4-3-5 與 3-4-1-5 兩級，騰出空間給 1-4-4-4。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="28" t="inlineStr">
+        <is>
+          <t>本表所列的修訂已就地套用於表 3、4、8、9；表 9 中標示「F舊」的六列為被摒棄的原 F 分支設計，僅供對照。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="28" t="inlineStr">
+        <is>
+          <t>書中未交代原本走 F 分支的「4張♠ + 5張以上♦、高限」牌型改走哪一條路線——這是原書留下的空白，不是本表的遺漏。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3652,7 +4330,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>雙重含義。接力序列（逼叫進局）的開始，或者是持有至少4張♥和6個以上大牌點的自然叫，和標準精確一樣。</t>
+          <t>雙重含義。接力序列（逼叫進局）的開始，或者是持有至少4張♥和7個以上大牌點的自然叫，和標準精確一樣。</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -3669,7 +4347,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>自然叫，至少4張♠，6個以上大牌點。</t>
+          <t>自然叫，至少4張♠，7個以上大牌點。</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -3686,7 +4364,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>6-11大牌點，通常無四張高花。</t>
+          <t>7-12大牌點，通常無四張高花。</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -3737,7 +4415,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>6張套，5-8個大牌點。（我們不採用強跳應叫，因為這種牌可以使用接力序列）</t>
+          <t>6張套，6-9個大牌點。（我們不採用強跳應叫，因為這種牌可以使用接力序列）</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -3754,7 +4432,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>邀叫牌力，10-13個大牌點，無四張高花。如果此前已經 pass 過，而且己方無局（我們使用10-12點的弱無將），2NT 則表示雙低花。</t>
+          <t>邀叫牌力，11-14個大牌點，無四張高花。如果此前已經 pass 過，而且己方無局（我們使用10-12點的弱無將），2NT 則表示雙低花。</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -3771,7 +4449,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>邀叫，通常至少6張好套，10個左右大牌點。</t>
+          <t>邀叫，通常至少6張好套，11個左右大牌點。</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -3812,7 +4490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3833,7 +4511,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>1♦ – 1♥ ； ？　（除 1♥ 外所有叫品都顯示 16-19 大牌點；前五種涵蓋 1♦ 開叫 90% 的情況）</t>
+          <t>1♦ – 1♥ ； ？　（所有再叫都在 1♦ 開叫的 10-14 大牌點範圍內；前五種涵蓋 1♦ 開叫 90% 的情況）</t>
         </is>
       </c>
     </row>
@@ -4042,7 +4720,7 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>4張以上♠+5張以上♦，高限</t>
+          <t>【第十一章修訂】4-4-4-1牌型，有4張♥，高限。（原含義「4張以上♠+5張以上♦，高限」已摒棄）</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
@@ -4052,7 +4730,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>54Pick-up</t>
+          <t>接力</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -4299,12 +4977,20 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>【第十一章修訂】F 分支的 2♠ 已改為 4441（4張♥）高限——因為新增的 2♦ 開叫把 4441 牌型全部推給了 1♦ 開叫。詳見「13.第十一章修訂」。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4316,7 +5002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4432,7 +5118,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>4張♠+6張以上♦，13-15大牌點</t>
+          <t>4張♠+6張以上♦，13-14大牌點</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -4455,7 +5141,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>4-2-5-2分佈，13-15大牌點</t>
+          <t>4-2-5-2分佈，13-14大牌點</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
@@ -4478,7 +5164,7 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>4-1-5-3分佈，13-15大牌點</t>
+          <t>4-1-5-3分佈，13-14大牌點</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
@@ -4501,7 +5187,7 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>4-3-5-1分佈，13-15大牌點</t>
+          <t>4-3-5-1分佈，13-14大牌點</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
@@ -4551,7 +5237,7 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>4-0-5-4分佈，13-15大牌點</t>
+          <t>4-0-5-4分佈，13-14大牌點</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
@@ -4590,94 +5276,214 @@
       <c r="E13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>2♠</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>2張♥，低花3-4或4-3</t>
-        </is>
-      </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>▸ 2♠</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>【修訂B】4張♠ + 1或2張♥。（原含義「2張♥，低花3-4或4-3」已取代）</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>2NT</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>接力</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>以下 4 列為 2♠ 之後的子接力</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　3♣</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>4-2-3-4</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>3♦</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>第十一章新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　3♦</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>4-2-4-3</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>3♥</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>第十一章新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　3♥</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>4-1-4-4，低限</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>3♠</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>第十一章新增（4441 併入）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　3♠</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>4-1-4-4，高限</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>4♣</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>第十一章新增（4441 併入）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>2NT</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>4-3-3-3分佈</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>3♣</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>3♣</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>4張♠+5張♣</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>3♦</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Sidestep</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>2NT</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>4-3-3-3分佈</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>3♣</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>3♣</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>4張♠+5張♣</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>3♦</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>Sidestep</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>＊）此時你不可能是高限（13-15點），否則你應該在 1♥ 接力後再叫 2♠。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>＊）此時你不可能是高限（13-14點），否則你應該在 1♥ 接力後再叫 2♠。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>藍底列為上層答叫，黃底列為其子接力答叫。</t>
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>【第十一章修訂B】2♠ 改為「4張♠＋1或2張♥」，把 4-1-4-4（♥單張）的 4441 牌型收進 A 分支——修訂A 的三個答叫都含4張♥，接不到這一型。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A24:E24"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A22:E22"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5463,7 +6269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5522,52 +6328,56 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>2NT</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>4張♠</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>▸ 2NT</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>【修訂C】4張♥ + 4張♠。（原含義「4張♠」已取代）</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>3♣</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Sidestep</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr"/>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>接力</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>以下 4 列為 2NT 之後的子接力</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>▸ 3♣</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>4張♥+4張以上♣</t>
-        </is>
-      </c>
-      <c r="C6" s="17" t="inlineStr">
-        <is>
-          <t>3♦</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>一種新的接力</t>
-        </is>
-      </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>以下 5 列為 3♣ 之後的子接力</t>
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　3♦</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>4-4-2-3</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>3♥</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>第十一章新增</t>
         </is>
       </c>
     </row>
@@ -5579,7 +6389,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>2-4-3-4</t>
+          <t>4-4-3-2</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -5592,7 +6402,11 @@
           <t>CRASH</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr"/>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>第十一章新增</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
@@ -5602,7 +6416,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>3-4-2-4</t>
+          <t>4-4-1-4，低限</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
@@ -5615,7 +6429,11 @@
           <t>CRASH</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr"/>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>第十一章新增（4441 併入）</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
@@ -5625,12 +6443,12 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>2-4-2-5</t>
+          <t>4-4-4-1，低限</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>4♦</t>
+          <t>4♣</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -5638,45 +6456,53 @@
           <t>CRASH</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr"/>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>第十一章新增（4441 併入）</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　4♣</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>1-4-3-5</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t>4♠</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr"/>
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>▸ 3♣</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>4張♥+4張以上♣　【修訂D：叫品不變，答叫階梯改寫】</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>3♦</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>一種新的接力</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>以下 4 列為 3♣ 之後的子接力</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">　4♦</t>
+          <t xml:space="preserve">　3♥</t>
         </is>
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>3-4-1-5</t>
+          <t>2-4-3-4</t>
         </is>
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
-          <t>4♠</t>
+          <t>3♠</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -5687,41 +6513,37 @@
       <c r="E11" s="19" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>▸ 3♦</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>4張♥+5張以上♦</t>
-        </is>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
-        <is>
-          <t>3♥</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>一種新的接力</t>
-        </is>
-      </c>
-      <c r="E12" s="16" t="inlineStr">
-        <is>
-          <t>以下 6 列為 3♦ 之後的子接力</t>
-        </is>
-      </c>
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　3♠</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>3-4-2-4</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>4♣</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">　3♠</t>
+          <t xml:space="preserve">　3NT</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>4張♥+6張以上♦</t>
+          <t>1-4-4-4，低限</t>
         </is>
       </c>
       <c r="C13" s="20" t="inlineStr">
@@ -5731,25 +6553,29 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Sidestep</t>
-        </is>
-      </c>
-      <c r="E13" s="19" t="inlineStr"/>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>第十一章新增（4441 併入）</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">　3NT</t>
+          <t xml:space="preserve">　4♣</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>2-4-5-2</t>
+          <t>2-4-2-5</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>4♣</t>
+          <t>4♦</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
@@ -5757,50 +6583,58 @@
           <t>CRASH</t>
         </is>
       </c>
-      <c r="E14" s="19" t="inlineStr"/>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>原為第3級，順延一級</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　4♣</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>1-4-5-3</t>
-        </is>
-      </c>
-      <c r="C15" s="20" t="inlineStr">
-        <is>
-          <t>4♦</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-      <c r="E15" s="19" t="inlineStr"/>
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>▸ 3♦</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>4張♥+5張以上♦</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>3♥</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>一種新的接力</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>以下 6 列為 3♦ 之後的子接力</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">　4♦</t>
+          <t xml:space="preserve">　3♠</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>3-4-5-1</t>
+          <t>4張♥+6張以上♦</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>4♠</t>
+          <t>4♣</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>CRASH</t>
+          <t>Sidestep</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr"/>
@@ -5808,17 +6642,17 @@
     <row r="17">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">　4♥</t>
+          <t xml:space="preserve">　3NT</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>0-4-5-4</t>
+          <t>2-4-5-2</t>
         </is>
       </c>
       <c r="C17" s="20" t="inlineStr">
         <is>
-          <t>4♠</t>
+          <t>4♣</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -5831,107 +6665,192 @@
     <row r="18">
       <c r="A18" s="18" t="inlineStr">
         <is>
+          <t xml:space="preserve">　4♣</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>1-4-5-3</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>4♦</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　4♦</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>3-4-5-1</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>4♠</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　4♥</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>0-4-5-4</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>4♠</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
           <t xml:space="preserve">　4♠</t>
         </is>
       </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>4-4-5-0</t>
         </is>
       </c>
-      <c r="C18" s="20" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>4NT</t>
         </is>
       </c>
-      <c r="D18" s="19" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
       </c>
-      <c r="E18" s="19" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="E21" s="19" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>3♥</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>2-4-4-3</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
         <is>
           <t>3♠</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>3♠</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>3-4-4-2</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>4♣</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>3NT</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>3-4-3-3</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t>4♣</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>藍底列為上層答叫，黃底列為其子接力答叫。本分支是全章唯一有兩組巢狀子接力的。</t>
+      <c r="E24" s="11" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>藍底列為上層答叫，黃底列為其子接力答叫。本分支原本就有兩組巢狀子接力，第十一章又把 2NT 也變成一組。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>【第十一章修訂C】2NT 由「4張♠」改為「4張♥+4張♠」，收進 4-4-1-4 與 4-4-4-1（皆低限）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>【第十一章修訂D】3♣ 的階梯在第3級插入 1-4-4-4（低限），2-4-2-5 順延到第4級；原本的 4♣ = 1-4-3-5 與 4♦ = 3-4-1-5 兩級取消。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="A26:E26"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A28:E28"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A27:E27"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5944,7 +6863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6010,7 +6929,7 @@
       <c r="B5" s="19" t="inlineStr">
         <is>
           <t>1♦–1♥；2♠–2NT；？
-2♠ = 4張以上♠+5張以上♦，高限</t>
+【第十一章修訂A】2♠ = 4-4-4-1牌型，有4張♥，高限</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
@@ -6020,7 +6939,7 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>4張♠+6張以上♦</t>
+          <t>4-4-4-1，高限（♣單張）</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -6030,7 +6949,7 @@
       </c>
       <c r="F5" s="19" t="inlineStr">
         <is>
-          <t>Sidestep</t>
+          <t>CRASH</t>
         </is>
       </c>
     </row>
@@ -6048,7 +6967,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>4-2-5-2</t>
+          <t>4-4-1-4，高限（♦單張）</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
@@ -6076,7 +6995,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>4-1-5-3</t>
+          <t>1-4-4-4，高限（♠單張）</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -6091,320 +7010,325 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr"/>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>3♠</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>4-3-5-1</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>4♣</t>
-        </is>
-      </c>
-      <c r="F8" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>F舊</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>（已摒棄）1♦–1♥；2♠–2NT；？
+原 2♠ = 4張以上♠+5張以上♦，高限</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>3♣</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>4張♠+6張以上♦</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>3♦</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>Sidestep</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>F舊</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr"/>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>3NT</t>
+          <t>3♦</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>5張♠+6張以上♦</t>
+          <t>4-2-5-2</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>4♣</t>
+          <t>3♥</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Sidestep</t>
+          <t>CRASH</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>F舊</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr"/>
       <c r="C10" s="10" t="inlineStr">
         <is>
+          <t>3♥</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>4-1-5-3</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>3♠</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>F舊</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr"/>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>3♠</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>4-3-5-1</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
           <t>4♣</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>F舊</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr"/>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>3NT</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>5張♠+6張以上♦</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>4♣</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Sidestep</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>F舊</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr"/>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>4♣</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>4-0-5-4</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>4♦</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>1♦–1♥；2NT–3♣；？
 2NT = 6張♦，高限</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>3♦</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>6-3-2-2</t>
         </is>
       </c>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>3♥</t>
         </is>
       </c>
-      <c r="F11" s="19" t="inlineStr">
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>Sidestep</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr"/>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr"/>
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>3♥</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>3-3-6-1</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>3♠</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr"/>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr"/>
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>3♠</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>3-1-6-3</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>4♣</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F16" s="11" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr"/>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr"/>
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>3NT</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>1-3-6-3</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>4♣</t>
         </is>
       </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>1♦–1♥；3♥–3♠；？
 3♥ = 4張以上♥+5張以上♦，高限</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>3NT</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>4張♥+6張以上♦</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>4♣</t>
         </is>
       </c>
-      <c r="F15" s="19" t="inlineStr">
+      <c r="F18" s="19" t="inlineStr">
         <is>
           <t>Sidestep</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr"/>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>4♣</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>2-4-5-2</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr">
-        <is>
-          <t>4♦</t>
-        </is>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr"/>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>4♦</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>1-4-5-3</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>4♠</t>
-        </is>
-      </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr"/>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>4♥</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>3-4-5-1</t>
-        </is>
-      </c>
-      <c r="E18" s="13" t="inlineStr">
-        <is>
-          <t>4♠</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
         </is>
       </c>
     </row>
@@ -6417,137 +7341,137 @@
       <c r="B19" s="11" t="inlineStr"/>
       <c r="C19" s="10" t="inlineStr">
         <is>
+          <t>4♣</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>2-4-5-2</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>4♦</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr"/>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>4♦</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>1-4-5-3</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
           <t>4♠</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr"/>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>4♥</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>3-4-5-1</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>4♠</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr"/>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>4♠</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>5張♥+6張以上♦</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E22" s="13" t="inlineStr">
         <is>
           <t>4NT</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>Blackwood　＊</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B23" s="19" t="inlineStr">
         <is>
           <t>1♦–1♥；3♠–4♣；？
 3♠ = 爆裂叫（♠單缺），4張以上♥+5張以上♦</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>4♦</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>1-4-5-3</t>
         </is>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E23" s="20" t="inlineStr">
         <is>
           <t>4♠</t>
         </is>
       </c>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr"/>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>4♥</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>0-4-5-4</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>4♠</t>
-        </is>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr"/>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>4♠</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>1-4-6-2</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>4NT</t>
-        </is>
-      </c>
-      <c r="F22" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr"/>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>4NT</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>0-4-6-3</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="inlineStr">
-        <is>
-          <t>5♣</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
@@ -6562,17 +7486,17 @@
       <c r="B24" s="11" t="inlineStr"/>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>5♣</t>
+          <t>4♥</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>1-4-7-1</t>
+          <t>0-4-5-4</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>5♠</t>
+          <t>4♠</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
@@ -6590,137 +7514,137 @@
       <c r="B25" s="11" t="inlineStr"/>
       <c r="C25" s="10" t="inlineStr">
         <is>
+          <t>4♠</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>1-4-6-2</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>4NT</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr"/>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>4NT</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>0-4-6-3</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>5♣</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr"/>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>5♣</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>1-4-7-1</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>5♠</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr"/>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
           <t>5♦</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>0-4-7-2</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="E28" s="13" t="inlineStr">
         <is>
           <t>5♠</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="18" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="B26" s="19" t="inlineStr">
+      <c r="B29" s="19" t="inlineStr">
         <is>
           <t>1♦–1♥；3NT–4♣；？
 3NT = 爆裂叫（♣單缺），其餘同 3♠</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>4♦</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D29" s="19" t="inlineStr">
         <is>
           <t>3-4-5-1</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="E29" s="20" t="inlineStr">
         <is>
           <t>4♠</t>
         </is>
       </c>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr"/>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>4♥</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>4-4-5-0</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>4NT</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>CRASH　＊＊</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr"/>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>4♠</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>2-4-6-1</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="inlineStr">
-        <is>
-          <t>4NT</t>
-        </is>
-      </c>
-      <c r="F28" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="B29" s="11" t="inlineStr"/>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>4NT</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>3-4-6-0</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>5♣</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="inlineStr">
+      <c r="F29" s="19" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
@@ -6735,22 +7659,22 @@
       <c r="B30" s="11" t="inlineStr"/>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>5♣</t>
+          <t>4♥</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>1-4-7-1</t>
+          <t>4-4-5-0</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>5♠</t>
+          <t>4NT</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>CRASH</t>
+          <t>CRASH　＊＊</t>
         </is>
       </c>
     </row>
@@ -6763,45 +7687,137 @@
       <c r="B31" s="11" t="inlineStr"/>
       <c r="C31" s="10" t="inlineStr">
         <is>
+          <t>4♠</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>2-4-6-1</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>4NT</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr"/>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>4NT</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>3-4-6-0</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>5♣</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr"/>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>5♣</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>1-4-7-1</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>5♠</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr"/>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
           <t>5♦</t>
         </is>
       </c>
-      <c r="D31" s="11" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>2-4-7-0</t>
         </is>
       </c>
-      <c r="E31" s="13" t="inlineStr">
+      <c r="E34" s="13" t="inlineStr">
         <is>
           <t>5♠</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr">
+      <c r="F34" s="11" t="inlineStr">
         <is>
           <t>CRASH</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>＊ 根據第三章的規則，4♠ 是詢問牌型的接力中最高階次的叫品，因此 4♠ 之後的 4NT 是黑木而非接力。</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>＊＊ 根據第三章的規則，任何在成局線上、且同伴至少保證四張的叫品都是止叫，所以此處只能用 4NT 做 CRASH 問叫。</t>
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>【第十一章修訂A】F 分支的 2♠ 已改為 4441（4張♥）高限，只剩三級答叫。標「F舊」的六列是被摒棄的原設計，保留供對照；書中未交代原本走 F 分支的「4張♠+5張以上♦高限」牌型改走哪裡。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A36:F36"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A37:F37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update 一方塊/一梅花/一無王 bidding tables from revised source workbooks
Reflects house rule that 1NT opens 10-12 HCP at any seat/vulnerability
and the resulting 1NT/1D/1C opening ladder.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/原始資料/一方塊開叫.xlsx
+++ b/原始資料/一方塊開叫.xlsx
@@ -681,7 +681,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>1♦ = 至少一張♦ + 10-14大牌點（家規下修 1 點；原書 11-15）。**低限 = 10-12 點，高限 = 13-14 點。**含義甚廣的多功能開叫，三種典型牌型：①至少5張♦的非均型牌　②均型牌但點力不在1NT範圍　③雙低花套（6♣+5♦ 總是開1♦，有時6♣+4♦ 也開1♦）。</t>
+          <t>1♦ = 至少一張♦ + 10-14大牌點（家規下修 1 點；原書 11-15）。**低限 = 10-12 點，高限 = 13-14 點。**均型牌的開叫階梯：10-12 → 1NT；13-14 → 1♦；15以上 → 1♣。含義甚廣的多功能開叫，三種典型牌型：①至少5張♦的非均型牌　②均型牌但點力不在1NT範圍　③雙低花套（6♣+5♦ 總是開1♦，有時6♣+4♦ 也開1♦）。</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>邀叫牌力，11-14個大牌點，無四張高花。如果此前已經 pass 過，而且己方無局（我們使用10-12點的弱無將），2NT 則表示雙低花。</t>
+          <t>邀叫牌力，11-14個大牌點，無四張高花。如果此前已經 pass 過，而且己方無局（我們的 1NT 開叫一律 10-12 點），2NT 則表示雙低花。</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Remove 示例牌張 and 示例叫序 sheets from bidding workbooks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/原始資料/一方塊開叫.xlsx
+++ b/原始資料/一方塊開叫.xlsx
@@ -17,9 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8.E分支(2♥)" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9.F-J分支" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10.非接力叫牌" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11.示例牌張" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12.示例叫序" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13.第十一章修訂" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11.第十一章修訂" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -628,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -649,6 +647,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1000,74 +999,50 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>11. 示例牌張</t>
+          <t>11. 第十一章修訂</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>例1–例6 的持牌、局況與結果評論。</t>
+          <t>★ 第十一章對本章的四處改寫（修訂A–D）新舊對照。表3、4、8、9 均已就地更新。</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>12. 示例叫序</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>例1–例6 的完整叫序，逐叫列出。</t>
-        </is>
-      </c>
+      <c r="A36" s="4" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>13. 第十一章修訂</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>★ 第十一章對本章的四處改寫（修訂A–D）新舊對照。表3、4、8、9 均已就地更新。</t>
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>★ 第十一章的影響</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>說明</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr"/>
-      <c r="B38" s="5" t="inlineStr"/>
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>為什麼要改</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>第十一章新增了「2♦ ＝ 4-8點、5張高花+4張低花」的選擇性開叫。這使得 4-4-4-1 牌型不得不全部歸給 1♦ 開叫，原有的接力設計容納不下，因此有了修訂 A～D 四處改寫。</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>★ 第十一章的影響</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>說明</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>為什麼要改</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>第十一章新增了「2♦ ＝ 4-8點、5張高花+4張低花」的選擇性開叫。這使得 4-4-4-1 牌型不得不全部歸給 1♦ 開叫，原有的接力設計容納不下，因此有了修訂 A～D 四處改寫。</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>改了哪四處</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>A：表3／表9 的 F分支 2♠ 改為「4441、有4張♥、高限」。
 B：表4 A分支的 2♠ 改為「4張♠+1或2張♥」，收 4-1-4-4。
@@ -1327,2402 +1302,6 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="62" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>叫牌示例：持牌、局況與結果</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>例號</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>出處</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>局況／發牌</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>方位</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>♠</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>♥</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>♦</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>♣</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>最終定約</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>評論</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t>例1</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>某次對式賽的第一副牌</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="inlineStr">
-        <is>
-          <t>雙無局，南發牌</t>
-        </is>
-      </c>
-      <c r="D4" s="20" t="inlineStr">
-        <is>
-          <t>北 Glenn</t>
-        </is>
-      </c>
-      <c r="E4" s="23" t="inlineStr">
-        <is>
-          <t>A8752</t>
-        </is>
-      </c>
-      <c r="F4" s="23" t="inlineStr">
-        <is>
-          <t>KQJ3</t>
-        </is>
-      </c>
-      <c r="G4" s="23" t="inlineStr">
-        <is>
-          <t>AJ</t>
-        </is>
-      </c>
-      <c r="H4" s="23" t="inlineStr">
-        <is>
-          <t>AJ</t>
-        </is>
-      </c>
-      <c r="I4" s="20" t="inlineStr">
-        <is>
-          <t>7NT</t>
-        </is>
-      </c>
-      <c r="J4" s="19" t="inlineStr">
-        <is>
-          <t>由於 Glenn 手裡持有♥KQ，因此他知道 Ulf 的K和Q都在低花上，於是很容易數出13墩牌。牌的配合如此之好，北家的3個J居然都派上了用場。（+11 IMP）</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>例1</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>南 Ulf</t>
-        </is>
-      </c>
-      <c r="E5" s="24" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="F5" s="24" t="inlineStr">
-        <is>
-          <t>A52</t>
-        </is>
-      </c>
-      <c r="G5" s="24" t="inlineStr">
-        <is>
-          <t>KQ85</t>
-        </is>
-      </c>
-      <c r="H5" s="24" t="inlineStr">
-        <is>
-          <t>KQ73</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr"/>
-      <c r="J5" s="11" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>例2</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>橋牌世界叫牌挑戰賽</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>雙有局，東發牌</t>
-        </is>
-      </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E6" s="23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="inlineStr">
-        <is>
-          <t>KJ98742</t>
-        </is>
-      </c>
-      <c r="G6" s="23" t="inlineStr">
-        <is>
-          <t>AQ98</t>
-        </is>
-      </c>
-      <c r="H6" s="23" t="inlineStr">
-        <is>
-          <t>K5</t>
-        </is>
-      </c>
-      <c r="I6" s="20" t="inlineStr">
-        <is>
-          <t>7♦</t>
-        </is>
-      </c>
-      <c r="J6" s="19" t="inlineStr">
-        <is>
-          <t>典型的改接力叫牌為自然叫牌的例子：沒有配合，且西家有一可能減值的缺門。關鍵是東的 4♣ 扣叫，表示持有♣而否認有♠控制。由於東的低花確定是4-5，西便清楚他的高花是2-2。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>例2</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>東 Geir Helgemo</t>
-        </is>
-      </c>
-      <c r="E7" s="24" t="inlineStr">
-        <is>
-          <t>85</t>
-        </is>
-      </c>
-      <c r="F7" s="24" t="inlineStr">
-        <is>
-          <t>A6</t>
-        </is>
-      </c>
-      <c r="G7" s="24" t="inlineStr">
-        <is>
-          <t>KJ65</t>
-        </is>
-      </c>
-      <c r="H7" s="24" t="inlineStr">
-        <is>
-          <t>A8643</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="inlineStr"/>
-      <c r="J7" s="11" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>例3</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>東西有局，南發牌</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E8" s="23" t="inlineStr">
-        <is>
-          <t>853</t>
-        </is>
-      </c>
-      <c r="F8" s="23" t="inlineStr">
-        <is>
-          <t>AK95</t>
-        </is>
-      </c>
-      <c r="G8" s="23" t="inlineStr">
-        <is>
-          <t>KQ9765</t>
-        </is>
-      </c>
-      <c r="H8" s="23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I8" s="20" t="inlineStr">
-        <is>
-          <t>6♦</t>
-        </is>
-      </c>
-      <c r="J8" s="19" t="inlineStr">
-        <is>
-          <t>5♣ 毫無疑問顯示缺門，因為此前的 3NT 是爆裂叫。5♠ 則是大滿貫試探，因為已經跨過了 5♦ 的成局線。如果西還持有♥Q或♠K，則會接受邀請並叫 5NT 核實將牌套質量。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>例3</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>東 Ulf</t>
-        </is>
-      </c>
-      <c r="E9" s="24" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="F9" s="24" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
-      </c>
-      <c r="G9" s="24" t="inlineStr">
-        <is>
-          <t>A1042</t>
-        </is>
-      </c>
-      <c r="H9" s="24" t="inlineStr">
-        <is>
-          <t>AJ974</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="inlineStr"/>
-      <c r="J9" s="11" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>例4</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>雙有局，南發牌</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>北 Geir</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>AK74</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="inlineStr">
-        <is>
-          <t>AQJ7</t>
-        </is>
-      </c>
-      <c r="G10" s="23" t="inlineStr">
-        <is>
-          <t>K10</t>
-        </is>
-      </c>
-      <c r="H10" s="23" t="inlineStr">
-        <is>
-          <t>AQ9</t>
-        </is>
-      </c>
-      <c r="I10" s="20" t="inlineStr">
-        <is>
-          <t>6NT</t>
-        </is>
-      </c>
-      <c r="J10" s="19" t="inlineStr">
-        <is>
-          <t>對北歐梅花這是很容易的一手牌。北家持有23點，因此在南家開叫後可以放心大膽地使用問叫，唯一需要決定的是打大滿貫還是小滿貫。Geir 的叫牌全是接力（3♥、4♣ 和 5♥ 是 CRASH）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>例4</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>南 Glenn</t>
-        </is>
-      </c>
-      <c r="E11" s="24" t="inlineStr">
-        <is>
-          <t>10962</t>
-        </is>
-      </c>
-      <c r="F11" s="24" t="inlineStr">
-        <is>
-          <t>K4</t>
-        </is>
-      </c>
-      <c r="G11" s="24" t="inlineStr">
-        <is>
-          <t>AJ97</t>
-        </is>
-      </c>
-      <c r="H11" s="24" t="inlineStr">
-        <is>
-          <t>K64</t>
-        </is>
-      </c>
-      <c r="I11" s="13" t="inlineStr"/>
-      <c r="J11" s="11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>例5</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>東西有局，西發牌</t>
-        </is>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E12" s="23" t="inlineStr">
-        <is>
-          <t>Q96</t>
-        </is>
-      </c>
-      <c r="F12" s="23" t="inlineStr">
-        <is>
-          <t>J76</t>
-        </is>
-      </c>
-      <c r="G12" s="23" t="inlineStr">
-        <is>
-          <t>K1092</t>
-        </is>
-      </c>
-      <c r="H12" s="23" t="inlineStr">
-        <is>
-          <t>AK2</t>
-        </is>
-      </c>
-      <c r="I12" s="20" t="inlineStr">
-        <is>
-          <t>3NT</t>
-        </is>
-      </c>
-      <c r="J12" s="19" t="inlineStr">
-        <is>
-          <t>東家 Ulf 可以在 2♦ 後叫出 4NT 表示示量加叫。西家持有高限13點且♦上有連張109無疑會接受邀請，但 Ulf 清楚在沒有配合且聯手不超過32個大牌點的情況下，滿貫的機會很小。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>例5</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>東 Ulf</t>
-        </is>
-      </c>
-      <c r="E13" s="24" t="inlineStr">
-        <is>
-          <t>KJ10</t>
-        </is>
-      </c>
-      <c r="F13" s="24" t="inlineStr">
-        <is>
-          <t>AK32</t>
-        </is>
-      </c>
-      <c r="G13" s="24" t="inlineStr">
-        <is>
-          <t>AQ</t>
-        </is>
-      </c>
-      <c r="H13" s="24" t="inlineStr">
-        <is>
-          <t>Q876</t>
-        </is>
-      </c>
-      <c r="I13" s="13" t="inlineStr"/>
-      <c r="J13" s="11" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>例6</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>1997歐錦賽 挪威對德國</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>南北有局，西發牌</t>
-        </is>
-      </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E14" s="23" t="inlineStr">
-        <is>
-          <t>KJ74</t>
-        </is>
-      </c>
-      <c r="F14" s="23" t="inlineStr">
-        <is>
-          <t>KQ2</t>
-        </is>
-      </c>
-      <c r="G14" s="23" t="inlineStr">
-        <is>
-          <t>QJ654</t>
-        </is>
-      </c>
-      <c r="H14" s="23" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="I14" s="20" t="inlineStr">
-        <is>
-          <t>6♦</t>
-        </is>
-      </c>
-      <c r="J14" s="19" t="inlineStr">
-        <is>
-          <t>Terje 接力詢問A、K、Q，發現西家有兩個K、3個Q，因此至少還應該有兩個J才能滿足高限開叫——這意味著西家的♦套必然是QJ領頭。於是 6♦ 必然比 6NT 優越得多。德國隊叫到 6NT 宕約，挪威得2 IMP。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>例6</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>東 Terje</t>
-        </is>
-      </c>
-      <c r="E15" s="24" t="inlineStr">
-        <is>
-          <t>983</t>
-        </is>
-      </c>
-      <c r="F15" s="24" t="inlineStr">
-        <is>
-          <t>AJ7</t>
-        </is>
-      </c>
-      <c r="G15" s="24" t="inlineStr">
-        <is>
-          <t>AK</t>
-        </is>
-      </c>
-      <c r="H15" s="24" t="inlineStr">
-        <is>
-          <t>AK1083</t>
-        </is>
-      </c>
-      <c r="I15" s="13" t="inlineStr"/>
-      <c r="J15" s="11" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F90"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>叫牌示例：完整叫序（逐叫）</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>例號</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>局況</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>序號</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>叫者</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>叫品</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>說明</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="25" t="inlineStr">
-        <is>
-          <t>例1</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>雙無局，南發牌</t>
-        </is>
-      </c>
-      <c r="C4" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="20" t="inlineStr">
-        <is>
-          <t>南 Ulf</t>
-        </is>
-      </c>
-      <c r="E4" s="18" t="inlineStr">
-        <is>
-          <t>1♦</t>
-        </is>
-      </c>
-      <c r="F4" s="19" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="26" t="inlineStr"/>
-      <c r="B5" s="11" t="inlineStr"/>
-      <c r="C5" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>北 Glenn</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>1♥</t>
-        </is>
-      </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>自然叫或逼局實力的接力叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="27" t="inlineStr"/>
-      <c r="B6" s="9" t="inlineStr"/>
-      <c r="C6" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>南 Ulf</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>1NT</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>均型牌，無四張高花，13-14大牌點（B分支）</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="26" t="inlineStr"/>
-      <c r="B7" s="11" t="inlineStr"/>
-      <c r="C7" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>北 Glenn</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>2♣</t>
-        </is>
-      </c>
-      <c r="F7" s="11" t="inlineStr">
-        <is>
-          <t>接力叫，逼局</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="27" t="inlineStr"/>
-      <c r="B8" s="9" t="inlineStr"/>
-      <c r="C8" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>南 Ulf</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>2♥</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>2-3-4-4牌型</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="26" t="inlineStr"/>
-      <c r="B9" s="11" t="inlineStr"/>
-      <c r="C9" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>北 Glenn</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>2♠</t>
-        </is>
-      </c>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="27" t="inlineStr"/>
-      <c r="B10" s="9" t="inlineStr"/>
-      <c r="C10" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>南 Ulf</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>2NT</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>1個A</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="26" t="inlineStr"/>
-      <c r="B11" s="11" t="inlineStr"/>
-      <c r="C11" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>北 Glenn</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>3♣</t>
-        </is>
-      </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="27" t="inlineStr"/>
-      <c r="B12" s="9" t="inlineStr"/>
-      <c r="C12" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>南 Ulf</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>3NT</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>2個低花或高花的K</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="26" t="inlineStr"/>
-      <c r="B13" s="11" t="inlineStr"/>
-      <c r="C13" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>北 Glenn</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>4♣</t>
-        </is>
-      </c>
-      <c r="F13" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="27" t="inlineStr"/>
-      <c r="B14" s="9" t="inlineStr"/>
-      <c r="C14" s="12" t="n">
-        <v>11</v>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>南 Ulf</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>4NT</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>2個低花或高花的Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="26" t="inlineStr"/>
-      <c r="B15" s="11" t="inlineStr"/>
-      <c r="C15" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>北 Glenn</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>7NT</t>
-        </is>
-      </c>
-      <c r="F15" s="11" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="28" t="inlineStr">
-        <is>
-          <t>註：B分支的教科書式用法：均型牌一叫定牌型，其餘全部空間拿來問 A→K→Q。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="25" t="inlineStr">
-        <is>
-          <t>例2</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>雙有局，東發牌</t>
-        </is>
-      </c>
-      <c r="C18" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>東 Geir</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>1♦</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="26" t="inlineStr"/>
-      <c r="B19" s="11" t="inlineStr"/>
-      <c r="C19" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>1♥</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>自然叫或逼局實力的接力叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="27" t="inlineStr"/>
-      <c r="B20" s="9" t="inlineStr"/>
-      <c r="C20" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>東 Geir</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>2♣</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="inlineStr">
-        <is>
-          <t>低花中至少有9張牌（C分支）</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="26" t="inlineStr"/>
-      <c r="B21" s="11" t="inlineStr"/>
-      <c r="C21" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>2♦</t>
-        </is>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
-        <is>
-          <t>接力叫，逼局</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="27" t="inlineStr"/>
-      <c r="B22" s="9" t="inlineStr"/>
-      <c r="C22" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>東 Geir</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>2♥</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>4張♦+5張♣</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="26" t="inlineStr"/>
-      <c r="B23" s="11" t="inlineStr"/>
-      <c r="C23" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>2♠</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Sidestep</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="27" t="inlineStr"/>
-      <c r="B24" s="9" t="inlineStr"/>
-      <c r="C24" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>東 Geir</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>2NT</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>低限開叫（C分支加一級的低限答叫）</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="26" t="inlineStr"/>
-      <c r="B25" s="11" t="inlineStr"/>
-      <c r="C25" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>3♥</t>
-        </is>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>自然叫！（脫離接力）</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="27" t="inlineStr"/>
-      <c r="B26" s="9" t="inlineStr"/>
-      <c r="C26" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>東 Geir</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>4♣</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="inlineStr">
-        <is>
-          <t>扣叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="26" t="inlineStr"/>
-      <c r="B27" s="11" t="inlineStr"/>
-      <c r="C27" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
-        <is>
-          <t>4♦</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>扣叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="27" t="inlineStr"/>
-      <c r="B28" s="9" t="inlineStr"/>
-      <c r="C28" s="12" t="n">
-        <v>11</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t>東 Geir</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>4♥</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>沒有更多可說的</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="26" t="inlineStr"/>
-      <c r="B29" s="11" t="inlineStr"/>
-      <c r="C29" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>4NT</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="inlineStr">
-        <is>
-          <t>羅馬關鍵張黑木問叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="27" t="inlineStr"/>
-      <c r="B30" s="9" t="inlineStr"/>
-      <c r="C30" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>東 Geir</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>5♥</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>2或5關鍵張，沒有♥Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="26" t="inlineStr"/>
-      <c r="B31" s="11" t="inlineStr"/>
-      <c r="C31" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>5NT</t>
-        </is>
-      </c>
-      <c r="F31" s="11" t="inlineStr">
-        <is>
-          <t>大滿貫試探叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="27" t="inlineStr"/>
-      <c r="B32" s="9" t="inlineStr"/>
-      <c r="C32" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t>東 Geir</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>6♦</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="inlineStr">
-        <is>
-          <t>我確實持有♦K</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="26" t="inlineStr"/>
-      <c r="B33" s="11" t="inlineStr"/>
-      <c r="C33" s="13" t="n">
-        <v>16</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E33" s="10" t="inlineStr">
-        <is>
-          <t>7♦</t>
-        </is>
-      </c>
-      <c r="F33" s="11" t="inlineStr">
-        <is>
-          <t>是改變將牌花色的時候了</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="27" t="inlineStr"/>
-      <c r="B34" s="9" t="inlineStr"/>
-      <c r="C34" s="12" t="n">
-        <v>17</v>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
-        <is>
-          <t>東 Geir</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="28" t="inlineStr">
-        <is>
-          <t>註：3♥ 後的 3♠ 有兩種可能含義：扣叫，或否認持有♠止張——後者可使 3NT 由正確的一方主打。</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="25" t="inlineStr">
-        <is>
-          <t>例3</t>
-        </is>
-      </c>
-      <c r="B37" s="19" t="inlineStr">
-        <is>
-          <t>東西有局，南發牌</t>
-        </is>
-      </c>
-      <c r="C37" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="20" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E37" s="18" t="inlineStr">
-        <is>
-          <t>1♦</t>
-        </is>
-      </c>
-      <c r="F37" s="19" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="26" t="inlineStr"/>
-      <c r="B38" s="11" t="inlineStr"/>
-      <c r="C38" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D38" s="13" t="inlineStr">
-        <is>
-          <t>東 Ulf</t>
-        </is>
-      </c>
-      <c r="E38" s="10" t="inlineStr">
-        <is>
-          <t>1♥</t>
-        </is>
-      </c>
-      <c r="F38" s="11" t="inlineStr">
-        <is>
-          <t>自然叫或逼局實力的接力叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="27" t="inlineStr"/>
-      <c r="B39" s="9" t="inlineStr"/>
-      <c r="C39" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D39" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>3NT</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>爆裂叫：短♣，4張♥+長♦，高限（J分支）</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="26" t="inlineStr"/>
-      <c r="B40" s="11" t="inlineStr"/>
-      <c r="C40" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D40" s="13" t="inlineStr">
-        <is>
-          <t>東 Ulf</t>
-        </is>
-      </c>
-      <c r="E40" s="10" t="inlineStr">
-        <is>
-          <t>4♦</t>
-        </is>
-      </c>
-      <c r="F40" s="11" t="inlineStr">
-        <is>
-          <t>自然叫，滿貫試探（脫離接力）</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="27" t="inlineStr"/>
-      <c r="B41" s="9" t="inlineStr"/>
-      <c r="C41" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D41" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>4♥</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="inlineStr">
-        <is>
-          <t>扣叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="26" t="inlineStr"/>
-      <c r="B42" s="11" t="inlineStr"/>
-      <c r="C42" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>東 Ulf</t>
-        </is>
-      </c>
-      <c r="E42" s="10" t="inlineStr">
-        <is>
-          <t>4♠</t>
-        </is>
-      </c>
-      <c r="F42" s="11" t="inlineStr">
-        <is>
-          <t>扣叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="27" t="inlineStr"/>
-      <c r="B43" s="9" t="inlineStr"/>
-      <c r="C43" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="D43" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>5♣</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="inlineStr">
-        <is>
-          <t>缺門</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="26" t="inlineStr"/>
-      <c r="B44" s="11" t="inlineStr"/>
-      <c r="C44" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t>東 Ulf</t>
-        </is>
-      </c>
-      <c r="E44" s="10" t="inlineStr">
-        <is>
-          <t>5♠</t>
-        </is>
-      </c>
-      <c r="F44" s="11" t="inlineStr">
-        <is>
-          <t>♠上有第一輪控制</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="27" t="inlineStr"/>
-      <c r="B45" s="9" t="inlineStr"/>
-      <c r="C45" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="D45" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>6♦</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="inlineStr">
-        <is>
-          <t>沒有額外牌力</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="26" t="inlineStr"/>
-      <c r="B46" s="11" t="inlineStr"/>
-      <c r="C46" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t>東 Ulf</t>
-        </is>
-      </c>
-      <c r="E46" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="F46" s="11" t="inlineStr">
-        <is>
-          <t>我也一樣</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="28" t="inlineStr">
-        <is>
-          <t>註：5♣ 顯示缺門而非控制，因為此前的 3NT 已是爆裂叫。</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="25" t="inlineStr">
-        <is>
-          <t>例4</t>
-        </is>
-      </c>
-      <c r="B49" s="19" t="inlineStr">
-        <is>
-          <t>雙有局，南發牌</t>
-        </is>
-      </c>
-      <c r="C49" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="20" t="inlineStr">
-        <is>
-          <t>南 Glenn</t>
-        </is>
-      </c>
-      <c r="E49" s="18" t="inlineStr">
-        <is>
-          <t>1♦</t>
-        </is>
-      </c>
-      <c r="F49" s="19" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="26" t="inlineStr"/>
-      <c r="B50" s="11" t="inlineStr"/>
-      <c r="C50" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D50" s="13" t="inlineStr">
-        <is>
-          <t>北 Geir</t>
-        </is>
-      </c>
-      <c r="E50" s="10" t="inlineStr">
-        <is>
-          <t>1♥</t>
-        </is>
-      </c>
-      <c r="F50" s="11" t="inlineStr">
-        <is>
-          <t>接力</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="27" t="inlineStr"/>
-      <c r="B51" s="9" t="inlineStr"/>
-      <c r="C51" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D51" s="12" t="inlineStr">
-        <is>
-          <t>南 Glenn</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>1♠</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>四張♠（A分支）</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="26" t="inlineStr"/>
-      <c r="B52" s="11" t="inlineStr"/>
-      <c r="C52" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D52" s="13" t="inlineStr">
-        <is>
-          <t>北 Geir</t>
-        </is>
-      </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>2♣</t>
-        </is>
-      </c>
-      <c r="F52" s="11" t="inlineStr">
-        <is>
-          <t>接力</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="27" t="inlineStr"/>
-      <c r="B53" s="9" t="inlineStr"/>
-      <c r="C53" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D53" s="12" t="inlineStr">
-        <is>
-          <t>南 Glenn</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>2♠</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="inlineStr">
-        <is>
-          <t>4-2-3-4 或 4-2-4-3 牌型</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="26" t="inlineStr"/>
-      <c r="B54" s="11" t="inlineStr"/>
-      <c r="C54" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="D54" s="13" t="inlineStr">
-        <is>
-          <t>北 Geir</t>
-        </is>
-      </c>
-      <c r="E54" s="10" t="inlineStr">
-        <is>
-          <t>2NT</t>
-        </is>
-      </c>
-      <c r="F54" s="11" t="inlineStr">
-        <is>
-          <t>Sidestep</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="27" t="inlineStr"/>
-      <c r="B55" s="9" t="inlineStr"/>
-      <c r="C55" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="D55" s="12" t="inlineStr">
-        <is>
-          <t>南 Glenn</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>3♦</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="inlineStr">
-        <is>
-          <t>4-2-4-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="26" t="inlineStr"/>
-      <c r="B56" s="11" t="inlineStr"/>
-      <c r="C56" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="D56" s="13" t="inlineStr">
-        <is>
-          <t>北 Geir</t>
-        </is>
-      </c>
-      <c r="E56" s="10" t="inlineStr">
-        <is>
-          <t>3♥</t>
-        </is>
-      </c>
-      <c r="F56" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="27" t="inlineStr"/>
-      <c r="B57" s="9" t="inlineStr"/>
-      <c r="C57" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="D57" s="12" t="inlineStr">
-        <is>
-          <t>南 Glenn</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>3♠</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="inlineStr">
-        <is>
-          <t>一個A</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="26" t="inlineStr"/>
-      <c r="B58" s="11" t="inlineStr"/>
-      <c r="C58" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="D58" s="13" t="inlineStr">
-        <is>
-          <t>北 Geir</t>
-        </is>
-      </c>
-      <c r="E58" s="10" t="inlineStr">
-        <is>
-          <t>4♣</t>
-        </is>
-      </c>
-      <c r="F58" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="27" t="inlineStr"/>
-      <c r="B59" s="9" t="inlineStr"/>
-      <c r="C59" s="12" t="n">
-        <v>11</v>
-      </c>
-      <c r="D59" s="12" t="inlineStr">
-        <is>
-          <t>南 Glenn</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>5♣</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="inlineStr">
-        <is>
-          <t>2個K，♣+♥ 或 ♦+♠</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="26" t="inlineStr"/>
-      <c r="B60" s="11" t="inlineStr"/>
-      <c r="C60" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="D60" s="13" t="inlineStr">
-        <is>
-          <t>北 Geir</t>
-        </is>
-      </c>
-      <c r="E60" s="10" t="inlineStr">
-        <is>
-          <t>5♥</t>
-        </is>
-      </c>
-      <c r="F60" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="27" t="inlineStr"/>
-      <c r="B61" s="9" t="inlineStr"/>
-      <c r="C61" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="D61" s="12" t="inlineStr">
-        <is>
-          <t>南 Glenn</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>5♠</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="inlineStr">
-        <is>
-          <t>沒有Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="26" t="inlineStr"/>
-      <c r="B62" s="11" t="inlineStr"/>
-      <c r="C62" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="D62" s="13" t="inlineStr">
-        <is>
-          <t>北 Geir</t>
-        </is>
-      </c>
-      <c r="E62" s="10" t="inlineStr">
-        <is>
-          <t>6NT</t>
-        </is>
-      </c>
-      <c r="F62" s="11" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="27" t="inlineStr"/>
-      <c r="B63" s="9" t="inlineStr"/>
-      <c r="C63" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="D63" s="12" t="inlineStr">
-        <is>
-          <t>南 Glenn</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="28" t="inlineStr">
-        <is>
-          <t>註：北家23點，可以一路問到底而不用擔心定約叫得過高。</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="25" t="inlineStr">
-        <is>
-          <t>例5</t>
-        </is>
-      </c>
-      <c r="B66" s="19" t="inlineStr">
-        <is>
-          <t>東西有局，西發牌</t>
-        </is>
-      </c>
-      <c r="C66" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="20" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E66" s="18" t="inlineStr">
-        <is>
-          <t>1♦</t>
-        </is>
-      </c>
-      <c r="F66" s="19" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="26" t="inlineStr"/>
-      <c r="B67" s="11" t="inlineStr"/>
-      <c r="C67" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D67" s="13" t="inlineStr">
-        <is>
-          <t>東 Ulf</t>
-        </is>
-      </c>
-      <c r="E67" s="10" t="inlineStr">
-        <is>
-          <t>1♥</t>
-        </is>
-      </c>
-      <c r="F67" s="11" t="inlineStr">
-        <is>
-          <t>自然叫或逼局實力的接力叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="27" t="inlineStr"/>
-      <c r="B68" s="9" t="inlineStr"/>
-      <c r="C68" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D68" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>1NT</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="inlineStr">
-        <is>
-          <t>均型牌，無4張高花，10-12點（B分支）</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="26" t="inlineStr"/>
-      <c r="B69" s="11" t="inlineStr"/>
-      <c r="C69" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D69" s="13" t="inlineStr">
-        <is>
-          <t>東 Ulf</t>
-        </is>
-      </c>
-      <c r="E69" s="10" t="inlineStr">
-        <is>
-          <t>2♣</t>
-        </is>
-      </c>
-      <c r="F69" s="11" t="inlineStr">
-        <is>
-          <t>接力叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="27" t="inlineStr"/>
-      <c r="B70" s="9" t="inlineStr"/>
-      <c r="C70" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D70" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E70" s="8" t="inlineStr">
-        <is>
-          <t>2♦</t>
-        </is>
-      </c>
-      <c r="F70" s="9" t="inlineStr">
-        <is>
-          <t>3-3-4-3牌型</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="26" t="inlineStr"/>
-      <c r="B71" s="11" t="inlineStr"/>
-      <c r="C71" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="D71" s="13" t="inlineStr">
-        <is>
-          <t>東 Ulf</t>
-        </is>
-      </c>
-      <c r="E71" s="10" t="inlineStr">
-        <is>
-          <t>3NT</t>
-        </is>
-      </c>
-      <c r="F71" s="11" t="inlineStr">
-        <is>
-          <t>沒有可打的滿貫</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="27" t="inlineStr"/>
-      <c r="B72" s="9" t="inlineStr"/>
-      <c r="C72" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="D72" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E72" s="8" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="F72" s="9" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="28" t="inlineStr">
-        <is>
-          <t>註：接力也可以用來確認「不要叫滿貫」——問清牌型後隨即停在 3NT。</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="25" t="inlineStr">
-        <is>
-          <t>例6</t>
-        </is>
-      </c>
-      <c r="B75" s="19" t="inlineStr">
-        <is>
-          <t>南北有局，西發牌</t>
-        </is>
-      </c>
-      <c r="C75" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D75" s="20" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E75" s="18" t="inlineStr">
-        <is>
-          <t>1♦</t>
-        </is>
-      </c>
-      <c r="F75" s="19" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="26" t="inlineStr"/>
-      <c r="B76" s="11" t="inlineStr"/>
-      <c r="C76" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D76" s="13" t="inlineStr">
-        <is>
-          <t>東 Terje</t>
-        </is>
-      </c>
-      <c r="E76" s="10" t="inlineStr">
-        <is>
-          <t>1♥</t>
-        </is>
-      </c>
-      <c r="F76" s="11" t="inlineStr">
-        <is>
-          <t>自然叫或逼局實力的接力叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="27" t="inlineStr"/>
-      <c r="B77" s="9" t="inlineStr"/>
-      <c r="C77" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D77" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E77" s="8" t="inlineStr">
-        <is>
-          <t>1♠</t>
-        </is>
-      </c>
-      <c r="F77" s="9" t="inlineStr">
-        <is>
-          <t>4張♠（A分支）</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="26" t="inlineStr"/>
-      <c r="B78" s="11" t="inlineStr"/>
-      <c r="C78" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D78" s="13" t="inlineStr">
-        <is>
-          <t>東 Terje</t>
-        </is>
-      </c>
-      <c r="E78" s="10" t="inlineStr">
-        <is>
-          <t>2♣</t>
-        </is>
-      </c>
-      <c r="F78" s="11" t="inlineStr">
-        <is>
-          <t>接力叫</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="27" t="inlineStr"/>
-      <c r="B79" s="9" t="inlineStr"/>
-      <c r="C79" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D79" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E79" s="8" t="inlineStr">
-        <is>
-          <t>2♦</t>
-        </is>
-      </c>
-      <c r="F79" s="9" t="inlineStr">
-        <is>
-          <t>4張♠+5張以上♦</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="26" t="inlineStr"/>
-      <c r="B80" s="11" t="inlineStr"/>
-      <c r="C80" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="D80" s="13" t="inlineStr">
-        <is>
-          <t>東 Terje</t>
-        </is>
-      </c>
-      <c r="E80" s="10" t="inlineStr">
-        <is>
-          <t>2♥</t>
-        </is>
-      </c>
-      <c r="F80" s="11" t="inlineStr">
-        <is>
-          <t>54Pick-up</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="27" t="inlineStr"/>
-      <c r="B81" s="9" t="inlineStr"/>
-      <c r="C81" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="D81" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E81" s="8" t="inlineStr">
-        <is>
-          <t>3♥</t>
-        </is>
-      </c>
-      <c r="F81" s="9" t="inlineStr">
-        <is>
-          <t>4-3-5-1牌型，高限</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="26" t="inlineStr"/>
-      <c r="B82" s="11" t="inlineStr"/>
-      <c r="C82" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="D82" s="13" t="inlineStr">
-        <is>
-          <t>東 Terje</t>
-        </is>
-      </c>
-      <c r="E82" s="10" t="inlineStr">
-        <is>
-          <t>3♠</t>
-        </is>
-      </c>
-      <c r="F82" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="27" t="inlineStr"/>
-      <c r="B83" s="9" t="inlineStr"/>
-      <c r="C83" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="D83" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E83" s="8" t="inlineStr">
-        <is>
-          <t>4♣</t>
-        </is>
-      </c>
-      <c r="F83" s="9" t="inlineStr">
-        <is>
-          <t>沒有A</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="26" t="inlineStr"/>
-      <c r="B84" s="11" t="inlineStr"/>
-      <c r="C84" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="D84" s="13" t="inlineStr">
-        <is>
-          <t>東 Terje</t>
-        </is>
-      </c>
-      <c r="E84" s="10" t="inlineStr">
-        <is>
-          <t>4♦</t>
-        </is>
-      </c>
-      <c r="F84" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="27" t="inlineStr"/>
-      <c r="B85" s="9" t="inlineStr"/>
-      <c r="C85" s="12" t="n">
-        <v>11</v>
-      </c>
-      <c r="D85" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E85" s="8" t="inlineStr">
-        <is>
-          <t>5♣</t>
-        </is>
-      </c>
-      <c r="F85" s="9" t="inlineStr">
-        <is>
-          <t>低花或高花2K</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="26" t="inlineStr"/>
-      <c r="B86" s="11" t="inlineStr"/>
-      <c r="C86" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="D86" s="13" t="inlineStr">
-        <is>
-          <t>東 Terje</t>
-        </is>
-      </c>
-      <c r="E86" s="10" t="inlineStr">
-        <is>
-          <t>5♥</t>
-        </is>
-      </c>
-      <c r="F86" s="11" t="inlineStr">
-        <is>
-          <t>CRASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="27" t="inlineStr"/>
-      <c r="B87" s="9" t="inlineStr"/>
-      <c r="C87" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="D87" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E87" s="8" t="inlineStr">
-        <is>
-          <t>5♠</t>
-        </is>
-      </c>
-      <c r="F87" s="9" t="inlineStr">
-        <is>
-          <t>0或3個Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="26" t="inlineStr"/>
-      <c r="B88" s="11" t="inlineStr"/>
-      <c r="C88" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="D88" s="13" t="inlineStr">
-        <is>
-          <t>東 Terje</t>
-        </is>
-      </c>
-      <c r="E88" s="10" t="inlineStr">
-        <is>
-          <t>6♦</t>
-        </is>
-      </c>
-      <c r="F88" s="11" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="27" t="inlineStr"/>
-      <c r="B89" s="9" t="inlineStr"/>
-      <c r="C89" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="D89" s="12" t="inlineStr">
-        <is>
-          <t>西 Glenn</t>
-        </is>
-      </c>
-      <c r="E89" s="8" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="F89" s="9" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="28" t="inlineStr">
-        <is>
-          <t>註：問完 A、K、Q 後用「高限開叫還缺幾點」反推出西家的♦套必是 QJ 領頭，因此選 6♦ 而非 6NT。</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A73:F73"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A47:F47"/>
-    <mergeCell ref="A90:F90"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="A64:F64"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>